<commit_message>
Update report: 동면 20260318_20260325
</commit_message>
<xml_diff>
--- a/shucle_report/동면/20260318_20260325/report_동면_20260318_20260325.xlsx
+++ b/shucle_report/동면/20260318_20260325/report_동면_20260318_20260325.xlsx
@@ -55,13 +55,13 @@
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
-      <color rgb="001565C0"/>
+      <color rgb="00D32F2F"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
-      <color rgb="00D32F2F"/>
+      <color rgb="001565C0"/>
       <sz val="9"/>
     </font>
     <font>
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>분석기간: 2026.03.18 ~ 03.25 | 비교기간: 2026.03.11 ~ 03.17 | 생성: 2026-03-26 14:48 | 차트: 124개</t>
+          <t>분석기간: 2026.03.18 ~ 03.25 | 비교기간: 2026.03.11 ~ 03.17 | 생성: 2026-03-26 15:08 | 차트: 124개</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.4건</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -592,17 +592,17 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-1.1건</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>-14.4%</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>감소</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.0건</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -629,17 +629,17 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+0.2건</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+2.8%</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>유지</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.6명</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -666,17 +666,17 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+0.7명</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+7.6%</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>유지</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
           <t>-21.1%</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>⚠ 감소</t>
         </is>
@@ -915,7 +915,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>68.7%</t>
+          <t>63.1%</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -925,12 +925,12 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>-0.5%p</t>
+          <t>+5.0%p</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>+7.9%</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1044,7 +1044,7 @@
           <t>-20.6%</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>⚠ 감소</t>
         </is>
@@ -1081,7 +1081,7 @@
           <t>-67.9%</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>⚠ 감소</t>
         </is>
@@ -1104,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1126,7 +1126,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>▼ DAU (일간 활성 회원) (-20.6%)</t>
+          <t>▼ 실시간 호출 건수(일평균) (-14.4%)</t>
         </is>
       </c>
     </row>
@@ -1170,310 +1170,614 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>DAU (일간 활성 회원)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>WAU (주간 활성 회원)</t>
+          <t>가호출 수(일평균)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>-2.6</t>
+          <t>-5.9</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>-72.2%</t>
+          <t>-52.4%</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>3.6→1.0명 감소</t>
+          <t>가호출/실호출 동반 감소</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>DAU (일간 활성 회원)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>신규 지역 회원(일평균)</t>
+          <t>배차실패 건수(일평균)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>-1.8</t>
+          <t>-0.8</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>-67.9%</t>
+          <t>-83.3%</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>신규 0.8명/일 (68% 감소)</t>
+          <t>배차실패 건수 83% 감소</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>DAU (일간 활성 회원)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>활성 회원 평균연령</t>
+          <t>호출취소 건수(일평균)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.4</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-100.0%</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>분석기간 데이터 없음</t>
+          <t>호출취소 건수 해소</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>DAU (일간 활성 회원)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>가호출 성공률</t>
+          <t>운행차량 대수</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>68.7%</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>68.2%</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-0.5%p</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>안정 유지, 영향 제한적</t>
+          <t>1대 유지, 증차 여지 없음</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>실시간 호출 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>전화 호출 비율</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>24.3%</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>21.1%</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>-3.3%p</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>-13.5%</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>전화 24→21%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>실시간 호출 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>앱 호출 비율</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>21.6%</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>18.4%</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>-3.2%p</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>-14.8%</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>앱 22→18%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>실시간 호출 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>현장 호출 비율</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>54.1%</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>60.5%</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>+6.5%p</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>+12.0%</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>현장 비중 61%로 주도적</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>▼ DAU (일간 활성 회원) (-20.6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>DAU (일간 활성 회원)</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>WAU (주간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>-2.6</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>-72.2%</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>3.6→1.0명 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>신규 지역 회원(일평균)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>-1.8</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>-67.9%</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>신규 0.8명/일 (68% 감소)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>활성 회원 평균연령</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>분석기간 데이터 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>63.1%</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>68.2%</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>+5.0%p</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>+7.9%</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>소폭 역방향 증가</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>평균 대기시간</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>-0.7</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>-21.1%</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>3.3→2.6분 감소</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>▼ 신규 지역 회원(일평균) (-67.9%)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>신규 지역 회원(일평균)</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>누적 지역 회원(일평균)</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>16.2</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>23.3</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>+7.1</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>+44.0%</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>누적 23명 (44% 증가)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>신규 지역 회원(일평균)</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>가호출 순 회원(일평균)</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>-0.9</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>-20.6%</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>4.2→3.3명 감소</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1486,7 +1790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1502,28 +1806,35 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>• 대기시간 개선: 3.3분 → 2.6분 (-21%) — 특히 03/24 상위10% 대기시간 9.7분으로 극단치 발생</t>
+          <t>• 수요 감소: 호출(-14%) 모두 하락 — 분석기간 운행 6일(03/18,03/19,03/20,03/23,03/24,03/25), 비교기간 5일</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>• 성장 지표 긍정적: DAU -21%, 신규회원 3→1명(-68%), 누적 30명</t>
+          <t>• 이동완료율 81.1% → 97.4% (+16.3%p): 호출 6건 중 6건 완료 (호출취소 0건, 배차실패 1건)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>• 호출당 평균 탑승객 1.7명: 동승 이용 활발</t>
+          <t>• 대기시간 개선: 3.3분 → 2.6분 (-21%) — 특히 03/24 상위10% 대기시간 9.7분으로 극단치 발생</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>• 수요 현황: 일평균 호출 6.3건, 이동완료 6.2건, 탑승객 10.3명</t>
+          <t>• 성장 지표 긍정적: DAU -21%, 신규회원 3→1명(-68%), 누적 30명</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>• 호출당 평균 탑승객 1.7명: 동승 이용 활발</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1563,7 +1874,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>▲ 대당 탑승객 수(일평균) (+7.6%)</t>
+          <t>▲ 이동완료 호출 건수(일평균) (+2.8%)</t>
         </is>
       </c>
     </row>
@@ -1607,1506 +1918,1855 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>이동완료 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(평일)</t>
+          <t>미탑승 건수(일평균)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>+0.7</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>+7.6%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>평일 10.3명 (8% 증가)</t>
+          <t>발생 없음</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>이동완료 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(주말)</t>
+          <t>호출취소 건수(일평균)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.4</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-100.0%</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>호출취소 건수 해소</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>이동완료 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
+          <t>배차실패 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>-0.8</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>-83.3%</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>배차실패 건수 83% 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>▲ 총 탑승객 수(일평균) (+7.6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>총 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
           <t>동승 인원 분포(일평균)</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>8.0</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>비교기간 데이터 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>대당 탑승객 수(일평균)</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>실시간 호출 건수(일평균)</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>6.3</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>비교기간 데이터 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>대당 탑승객 수(일평균)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>운행차량 대수</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>+0.0</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>1대 유지, 증차 여지 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>▼ 평균 대기시간 (-21.1%)</t>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>-1.6</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>-16.7%</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>감소 전환 (17%)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>세부지표</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>비교기간</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>분석기간</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>변동값</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>변동률</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>포인트</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>총 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>고령자(60+) 호출 비율</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>47.3%</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>77.8%</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>+30.5%p</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>+64.6%</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>고령자(60+) 비중 78%로 주도적</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>평균 대기시간</t>
+          <t>총 탑승객 수(일평균)</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>평균 대기시간(평일)</t>
+          <t>성인(20~50대) 호출 비율</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>41.8%</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>-0.7</t>
+          <t>-41.8%p</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>-21.1%</t>
+          <t>-100.0%</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>평일 2.6분 (21% 감소)</t>
+          <t>성인(20~50대) 42→0%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>평균 대기시간</t>
+          <t>총 탑승객 수(일평균)</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>평균 대기시간(주말)</t>
+          <t>어린이/청소년 호출 비율</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+11.2%p</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+102.2%</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>평균 대기시간</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>상위 10% 대기시간</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>7.4</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>-3.7</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>-33.5%</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>극단 대기 34% 감소</t>
+          <t>어린이/청소년 11→22%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>평균 대기시간</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>장시간 대기(30분+) 비율</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%p</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>변동 없음</t>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>▲ 대당 탑승객 수(일평균) (+7.6%)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>평균 대기시간</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>운행차량 대수</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>+0.0</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>1대 유지, 증차 여지 없음</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>평균 대기시간</t>
+          <t>대당 탑승객 수(일평균)</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
+          <t>대당 탑승객 수(평일)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>+0.7</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>+7.6%</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>평일 10.3명 (8% 증가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(주말)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>데이터 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>동승 인원 분포(일평균)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>-1.6</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>-16.7%</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>감소 전환 (17%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
           <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>비교기간 데이터 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>▲ 평균 우회비율 (+7.3%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>세부지표</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>비교기간</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>분석기간</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>변동값</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>변동률</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>포인트</t>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>-1.1</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>-14.4%</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>감소 전환 (14%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>평균 우회비율</t>
+          <t>대당 탑승객 수(일평균)</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>상위 10% 우회비율</t>
+          <t>운행차량 대수</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>+0.1</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>+4.8%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>1.6배 안정</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>평균 우회비율</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>평균 이동시간</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>9.5</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>8.7</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>-0.8</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>-8.2%</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>9.5→8.7분 감소</t>
+          <t>1대 유지, 증차 여지 없음</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>평균 우회비율</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>동승 인원 분포(일평균)</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>▼ 평균 대기시간 (-21.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>평균 대기시간</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>평균 대기시간(평일)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>-0.7</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>-21.1%</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>평일 2.6분 (21% 감소)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>평균 대기시간</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>평균 대기시간(주말)</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>비교기간 데이터 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>▼ 평균 이동시간 (-8.2%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>세부지표</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>비교기간</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>분석기간</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>변동값</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>변동률</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>포인트</t>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>데이터 없음</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>평균 이동시간</t>
+          <t>평균 대기시간</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>피크 시간대(15~17시) 이동시간</t>
+          <t>상위 10% 대기시간</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>8.6</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>-1.5</t>
+          <t>-3.7</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>-14.5%</t>
+          <t>-33.5%</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>10.1→8.6분 감소</t>
+          <t>극단 대기 34% 감소</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>평균 이동시간</t>
+          <t>평균 대기시간</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>비피크 시간대(8~10시) 이동시간</t>
+          <t>장시간 대기(30분+) 비율</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>12.6</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>-0.9</t>
+          <t>+0.0%p</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>-7.2%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>12.6→11.7분 감소</t>
+          <t>변동 없음</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>평균 이동시간</t>
+          <t>평균 대기시간</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>평균 우회비율</t>
+          <t>운행차량 대수</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>+0.1</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>+7.3%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>1.1→1.1배 증가</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>─ 운행차량 대수 (+0.0%)</t>
+          <t>1대 유지, 증차 여지 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>평균 대기시간</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>실시간 호출 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>-1.1</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>-14.4%</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>동반 감소 (14%)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>▲ 평균 우회비율 (+7.3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>운행차량 대수</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>일별 운행 차량 수</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>+0.0</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>0% 감소</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>운행차량 대수</t>
+          <t>평균 우회비율</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>근무 이행률</t>
+          <t>상위 10% 우회비율</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>-0.0</t>
+          <t>+0.1</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>+4.8%</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>1.0시간 유지</t>
+          <t>1.6배 안정</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>운행차량 대수</t>
+          <t>평균 우회비율</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>배차실패 건수(일평균)</t>
+          <t>평균 이동시간</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.8</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-8.2%</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>비교기간 데이터 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>▼ 대당 운행시간(일평균) (-1.5%)</t>
+          <t>9.5→8.7분 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>평균 우회비율</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>동승 인원 분포(일평균)</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>-1.6</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>-16.7%</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>감소 전환 (17%)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>▼ 평균 이동시간 (-8.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>대당 운행시간(일평균)</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>차량별 운행 시간</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>7.4</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>7.3</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>-0.1</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>-1.5%</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>안정 유지, 영향 제한적</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>대당 운행시간(일평균)</t>
+          <t>평균 이동시간</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>평균 근무시간</t>
+          <t>피크 시간대(15~17시) 이동시간</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>8.6</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>-0.1</t>
+          <t>-1.5</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>-14.5%</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>9.2시간 유지</t>
+          <t>10.1→8.6분 감소</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>대당 운행시간(일평균)</t>
+          <t>평균 이동시간</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>차량 대당 탑승객</t>
+          <t>비피크 시간대(8~10시) 이동시간</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>12.6</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>+0.7</t>
+          <t>-0.9</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>+7.6%</t>
+          <t>-7.2%</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>소폭 역방향 증가</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>▼ 가호출 성공률 (-0.7%)</t>
+          <t>12.6→11.7분 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>평균 이동시간</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>평균 우회비율</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>+0.1</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>+7.3%</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>1.1→1.1배 증가</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>─ 운행차량 대수 (+0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>세부지표</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>비교기간</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>분석기간</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>변동값</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>변동률</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>포인트</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>가호출 성공률</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>가호출 성공률(평일)</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>68.7%</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>68.2%</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>-0.5%p</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>-0.7%</t>
-        </is>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>평일 68% (1% 감소)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>가호출 성공률</t>
+          <t>운행차량 대수</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>가호출 성공률(주말)</t>
+          <t>일별 운행 차량 수</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>0% 감소</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>가호출 성공률</t>
+          <t>운행차량 대수</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>피크 시간대 가호출 성공률</t>
+          <t>근무 이행률</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.0</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.7%</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>1.0시간 유지</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>가호출 성공률</t>
+          <t>운행차량 대수</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>가호출 성공/실패 회원(일평균)</t>
+          <t>배차실패 건수(일평균)</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>-2.3</t>
+          <t>-0.8</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>-40.5%</t>
+          <t>-83.3%</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>5.6→3.3명 감소</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>가호출 성공률</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>운행차량 대수</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>+0.0</t>
-        </is>
-      </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>+0.0%</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>1대 유지, 증차 여지 없음</t>
+          <t>배차실패 건수 83% 감소</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>가호출 성공률</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>가호출 수(일평균)</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>-5.9</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>-52.4%</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>가호출 52% 감소</t>
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>▼ 대당 운행시간(일평균) (-1.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="inlineStr">
-        <is>
-          <t>▼ 대당 운행거리(일평균) (-0.5%)</t>
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>대당 운행시간(일평균)</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>차량별 운행 시간</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>-0.1</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>-1.5%</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>안정 유지, 영향 제한적</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>세부지표</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>비교기간</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>분석기간</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>변동값</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>변동률</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>포인트</t>
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>대당 운행시간(일평균)</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>평균 근무시간</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>-0.1</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>-0.7%</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>9.2시간 유지</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
+          <t>대당 운행시간(일평균)</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>차량 대당 탑승객</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>+0.7</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>+7.6%</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>소폭 역방향 증가</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>▲ 가호출 성공률 (+7.9%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률(평일)</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>63.1%</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>68.2%</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>+5.0%p</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>+7.9%</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>평일 68% (8% 증가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률(주말)</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>데이터 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>피크 시간대 가호출 성공률</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>데이터 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공/실패 회원(일평균)</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>-2.3</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>-40.5%</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>5.6→3.3명 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>운행차량 대수</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>+0.0</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>1대 유지, 증차 여지 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>가호출 성공률</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>가호출 수(일평균)</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>-5.9</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>-52.4%</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>가호출 52% 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>▼ 대당 운행거리(일평균) (-0.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
           <t>대당 운행거리(일평균)</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>일간 평균 대당 운행거리</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>78.2</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D68" s="7" t="inlineStr">
         <is>
           <t>77.8</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E68" s="7" t="inlineStr">
         <is>
           <t>-0.4</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>-0.5%</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>안정 유지, 영향 제한적</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>대당 운행거리(일평균)</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>비교기간 데이터 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>-1.1</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>-14.4%</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>동반 감소 (14%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
         <is>
           <t>대당 운행거리(일평균)</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B70" s="6" t="inlineStr">
         <is>
           <t>운행차량 대수</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C70" s="7" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D70" s="7" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E70" s="7" t="inlineStr">
         <is>
           <t>+0.0</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>+0.0%</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>1대 유지, 증차 여지 없음</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="A44:G44"/>
+  <mergeCells count="11">
+    <mergeCell ref="A66:G66"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:G9"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A45:G45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>